<commit_message>
Dashboard 2026-09-08 + файлы лотов
</commit_message>
<xml_diff>
--- a/vse-loti/339759366/spec-339759366.xlsx
+++ b/vse-loti/339759366/spec-339759366.xlsx
@@ -16,9 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.00&quot; ₽&quot;"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -60,15 +58,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -500,49 +496,33 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Труба стальная</t>
+          <t>плуатации. Значение характеристики не может изменяться участником закупки 2 Длина</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" s="2" t="n">
-        <v>1500</v>
+        <v>4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Погонный метр</t>
+          <t>м</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" s="3" t="n">
-        <v>1012455</v>
-      </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
-      </c>
-      <c r="G3" s="5" t="n">
-        <v>1012455</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>НМЦК из обоснования:</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>1012455</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Источник: preview.txt</t>
+          <t>Источник: Приложение № 2_РНМЦК_труба.docx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard 2026-09-11 + файлы лотов
</commit_message>
<xml_diff>
--- a/vse-loti/339759366/spec-339759366.xlsx
+++ b/vse-loti/339759366/spec-339759366.xlsx
@@ -547,16 +547,16 @@
         </is>
       </c>
       <c r="F2" s="4" t="n">
-        <v>6.93</v>
+        <v>5.993</v>
       </c>
       <c r="G2" s="5" t="n">
         <v>1012455</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>146097.4</v>
+        <v>146671.12</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>175316.88</v>
+        <v>176005.34</v>
       </c>
     </row>
     <row r="3">
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="F3" s="7" t="n">
-        <v>6.93</v>
+        <v>5.993</v>
       </c>
       <c r="G3" s="8" t="n">
         <v>1012455</v>

</xml_diff>